<commit_message>
Update 15-05-2026: Separada simulación en otro script
</commit_message>
<xml_diff>
--- a/datos_limpios/arg_avad_abs.xlsx
+++ b/datos_limpios/arg_avad_abs.xlsx
@@ -393,13 +393,13 @@
         </is>
       </c>
       <c r="C2">
-        <v>155905.0247732566</v>
+        <v>125792.8618224136</v>
       </c>
       <c r="D2">
-        <v>88041.71406785498</v>
+        <v>57834.21218639016</v>
       </c>
       <c r="E2">
-        <v>67923.50175899046</v>
+        <v>67946.157264448</v>
       </c>
     </row>
     <row r="3">
@@ -414,13 +414,13 @@
         </is>
       </c>
       <c r="C3">
-        <v>173705.7338406137</v>
+        <v>153879.2486412149</v>
       </c>
       <c r="D3">
-        <v>107633.8430202827</v>
+        <v>87835.29147578134</v>
       </c>
       <c r="E3">
-        <v>66034.7767830752</v>
+        <v>66049.30347332754</v>
       </c>
     </row>
     <row r="4">
@@ -435,13 +435,13 @@
         </is>
       </c>
       <c r="C4">
-        <v>147639.1175670573</v>
+        <v>105385.9049020076</v>
       </c>
       <c r="D4">
-        <v>86744.61785783361</v>
+        <v>44462.15581978112</v>
       </c>
       <c r="E4">
-        <v>60927.46132663983</v>
+        <v>60929.53742243133</v>
       </c>
     </row>
     <row r="5">
@@ -456,13 +456,13 @@
         </is>
       </c>
       <c r="C5">
-        <v>165930.3974909637</v>
+        <v>137892.1882338689</v>
       </c>
       <c r="D5">
-        <v>107351.7925429942</v>
+        <v>79316.69789186436</v>
       </c>
       <c r="E5">
-        <v>58535.8120627857</v>
+        <v>58558.67480076513</v>
       </c>
     </row>
     <row r="6">
@@ -477,13 +477,13 @@
         </is>
       </c>
       <c r="C6">
-        <v>208673.788464195</v>
+        <v>170390.7669132832</v>
       </c>
       <c r="D6">
-        <v>147577.4494629193</v>
+        <v>109322.7188045944</v>
       </c>
       <c r="E6">
-        <v>61056.43861018956</v>
+        <v>61057.07760437026</v>
       </c>
     </row>
     <row r="7">
@@ -498,13 +498,13 @@
         </is>
       </c>
       <c r="C7">
-        <v>231582.0394689974</v>
+        <v>208346.8612187625</v>
       </c>
       <c r="D7">
-        <v>170157.3172135107</v>
+        <v>146865.3848599756</v>
       </c>
       <c r="E7">
-        <v>61462.37787931033</v>
+        <v>61450.16767579936</v>
       </c>
     </row>
     <row r="8">
@@ -519,13 +519,13 @@
         </is>
       </c>
       <c r="C8">
-        <v>247483.0882392639</v>
+        <v>200120.6126092919</v>
       </c>
       <c r="D8">
-        <v>182098.1197097914</v>
+        <v>134741.3194329927</v>
       </c>
       <c r="E8">
-        <v>65386.44634457536</v>
+        <v>65391.22693517628</v>
       </c>
     </row>
     <row r="9">
@@ -540,13 +540,13 @@
         </is>
       </c>
       <c r="C9">
-        <v>335242.8112563242</v>
+        <v>304082.0420495539</v>
       </c>
       <c r="D9">
-        <v>264699.2551714047</v>
+        <v>233618.8578987021</v>
       </c>
       <c r="E9">
-        <v>70516.01823656166</v>
+        <v>70504.56489624894</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
calculo de AVD por complicación
</commit_message>
<xml_diff>
--- a/datos_limpios/arg_avad_abs.xlsx
+++ b/datos_limpios/arg_avad_abs.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:S13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -380,6 +380,76 @@
           <t>AVAD</t>
         </is>
       </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>AVD_total_micro</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>AVD_total_macro</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>AVD_sin_complicaciones</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>AVD_micro_neuropatia_p</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>AVD_micro_retinopatia_np</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>AVD_micro_retinopatia_p</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>AVD_micro_disf_erectil</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>AVD_micro_nefropatia</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>AVD_micro_ceguera</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>AVD_micro_amputacion</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>AVD_macro_claudicacion</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>AVD_macro_acv</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>AVD_macro_iam</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>AVD_macro_ic</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -396,10 +466,52 @@
         <v>67946.157264448</v>
       </c>
       <c r="D2">
-        <v>34855.49287611758</v>
+        <v>88058.22313981604</v>
       </c>
       <c r="E2">
-        <v>102778.7956897096</v>
+        <v>156024.0142917577</v>
+      </c>
+      <c r="F2">
+        <v>49171.27943042637</v>
+      </c>
+      <c r="G2">
+        <v>8662.93275596379</v>
+      </c>
+      <c r="H2">
+        <v>30224.01095342588</v>
+      </c>
+      <c r="I2">
+        <v>14295.24902569345</v>
+      </c>
+      <c r="J2">
+        <v>8359.667699395246</v>
+      </c>
+      <c r="K2">
+        <v>4163.452268280073</v>
+      </c>
+      <c r="L2">
+        <v>0</v>
+      </c>
+      <c r="M2">
+        <v>19029.94003712475</v>
+      </c>
+      <c r="N2">
+        <v>1674.740144241426</v>
+      </c>
+      <c r="O2">
+        <v>1648.230255691433</v>
+      </c>
+      <c r="P2">
+        <v>570.9374623726552</v>
+      </c>
+      <c r="Q2">
+        <v>4635.761725173016</v>
+      </c>
+      <c r="R2">
+        <v>3456.233568418117</v>
+      </c>
+      <c r="S2">
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -417,10 +529,52 @@
         <v>66049.30347332754</v>
       </c>
       <c r="D3">
-        <v>28530.59939633048</v>
+        <v>107768.5295173201</v>
       </c>
       <c r="E3">
-        <v>94582.40000056845</v>
+        <v>173807.3991852785</v>
+      </c>
+      <c r="F3">
+        <v>67381.63594192796</v>
+      </c>
+      <c r="G3">
+        <v>20453.65553385339</v>
+      </c>
+      <c r="H3">
+        <v>19933.23804153871</v>
+      </c>
+      <c r="I3">
+        <v>18619.08451818477</v>
+      </c>
+      <c r="J3">
+        <v>6552.57408909446</v>
+      </c>
+      <c r="K3">
+        <v>2870.959542846104</v>
+      </c>
+      <c r="L3">
+        <v>15989.78494238615</v>
+      </c>
+      <c r="M3">
+        <v>17026.57247247187</v>
+      </c>
+      <c r="N3">
+        <v>1506.318301422069</v>
+      </c>
+      <c r="O3">
+        <v>4816.342075522539</v>
+      </c>
+      <c r="P3">
+        <v>809.0352043863065</v>
+      </c>
+      <c r="Q3">
+        <v>8641.986996559439</v>
+      </c>
+      <c r="R3">
+        <v>11002.63333290765</v>
+      </c>
+      <c r="S3">
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -438,10 +592,52 @@
         <v>60929.53742243133</v>
       </c>
       <c r="D4">
-        <v>52577.5613899598</v>
+        <v>86675.6560383484</v>
       </c>
       <c r="E4">
-        <v>113501.9970194888</v>
+        <v>147596.3163216352</v>
+      </c>
+      <c r="F4">
+        <v>26369.30439279917</v>
+      </c>
+      <c r="G4">
+        <v>18092.85142698195</v>
+      </c>
+      <c r="H4">
+        <v>42213.50021856728</v>
+      </c>
+      <c r="I4">
+        <v>16977.77116995841</v>
+      </c>
+      <c r="J4">
+        <v>2695.240486787595</v>
+      </c>
+      <c r="K4">
+        <v>1662.204468060287</v>
+      </c>
+      <c r="L4">
+        <v>0</v>
+      </c>
+      <c r="M4">
+        <v>3593.675202013848</v>
+      </c>
+      <c r="N4">
+        <v>423.9626914012164</v>
+      </c>
+      <c r="O4">
+        <v>1016.450374577821</v>
+      </c>
+      <c r="P4">
+        <v>557.2111852204824</v>
+      </c>
+      <c r="Q4">
+        <v>10385.58050837481</v>
+      </c>
+      <c r="R4">
+        <v>7150.059733386663</v>
+      </c>
+      <c r="S4">
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -459,10 +655,52 @@
         <v>58558.67480076513</v>
       </c>
       <c r="D5">
-        <v>44213.45260004531</v>
+        <v>107374.6918651472</v>
       </c>
       <c r="E5">
-        <v>102749.5304014887</v>
+        <v>165955.097013882</v>
+      </c>
+      <c r="F5">
+        <v>55437.36642936451</v>
+      </c>
+      <c r="G5">
+        <v>23879.33146249985</v>
+      </c>
+      <c r="H5">
+        <v>28057.99397328282</v>
+      </c>
+      <c r="I5">
+        <v>21030.96696691602</v>
+      </c>
+      <c r="J5">
+        <v>2316.409301371934</v>
+      </c>
+      <c r="K5">
+        <v>3382.119896087782</v>
+      </c>
+      <c r="L5">
+        <v>11594.9609510793</v>
+      </c>
+      <c r="M5">
+        <v>13532.44141637856</v>
+      </c>
+      <c r="N5">
+        <v>1303.294736590552</v>
+      </c>
+      <c r="O5">
+        <v>2277.173160940362</v>
+      </c>
+      <c r="P5">
+        <v>553.5548607173778</v>
+      </c>
+      <c r="Q5">
+        <v>16086.61814483623</v>
+      </c>
+      <c r="R5">
+        <v>7239.158456946237</v>
+      </c>
+      <c r="S5">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -480,10 +718,52 @@
         <v>61057.07760437026</v>
       </c>
       <c r="D6">
-        <v>45587.23935596566</v>
+        <v>147645.0517066229</v>
       </c>
       <c r="E6">
-        <v>106628.7145917741</v>
+        <v>208709.025511501</v>
+      </c>
+      <c r="F6">
+        <v>82511.50334848286</v>
+      </c>
+      <c r="G6">
+        <v>26811.21545611159</v>
+      </c>
+      <c r="H6">
+        <v>38322.33290202846</v>
+      </c>
+      <c r="I6">
+        <v>28055.72407955932</v>
+      </c>
+      <c r="J6">
+        <v>14405.7143654849</v>
+      </c>
+      <c r="K6">
+        <v>7003.568742231339</v>
+      </c>
+      <c r="L6">
+        <v>0</v>
+      </c>
+      <c r="M6">
+        <v>30573.79211814593</v>
+      </c>
+      <c r="N6">
+        <v>798.5047332816767</v>
+      </c>
+      <c r="O6">
+        <v>1674.199309779689</v>
+      </c>
+      <c r="P6">
+        <v>1095.568165379696</v>
+      </c>
+      <c r="Q6">
+        <v>7234.923738659742</v>
+      </c>
+      <c r="R6">
+        <v>15105.74777246624</v>
+      </c>
+      <c r="S6">
+        <v>3374.975779605913</v>
       </c>
     </row>
     <row r="7">
@@ -501,10 +781,52 @@
         <v>61450.16767579936</v>
       </c>
       <c r="D7">
-        <v>31153.70149323768</v>
+        <v>170285.6923141014</v>
       </c>
       <c r="E7">
-        <v>92626.81542266223</v>
+        <v>231768.5951619562</v>
+      </c>
+      <c r="F7">
+        <v>114151.4432677223</v>
+      </c>
+      <c r="G7">
+        <v>32713.94159225322</v>
+      </c>
+      <c r="H7">
+        <v>23420.30745412581</v>
+      </c>
+      <c r="I7">
+        <v>29548.63250336926</v>
+      </c>
+      <c r="J7">
+        <v>9404.699049726914</v>
+      </c>
+      <c r="K7">
+        <v>13356.88810825615</v>
+      </c>
+      <c r="L7">
+        <v>27250.68677264273</v>
+      </c>
+      <c r="M7">
+        <v>30163.71340112469</v>
+      </c>
+      <c r="N7">
+        <v>462.2415305711813</v>
+      </c>
+      <c r="O7">
+        <v>3964.581902031427</v>
+      </c>
+      <c r="P7">
+        <v>976.4655353791384</v>
+      </c>
+      <c r="Q7">
+        <v>7734.653801042098</v>
+      </c>
+      <c r="R7">
+        <v>18496.17514922945</v>
+      </c>
+      <c r="S7">
+        <v>5506.647106602535</v>
       </c>
     </row>
     <row r="8">
@@ -522,10 +844,52 @@
         <v>65391.22693517628</v>
       </c>
       <c r="D8">
-        <v>59758.58100970614</v>
+        <v>181983.8557410124</v>
       </c>
       <c r="E8">
-        <v>125139.827683761</v>
+        <v>247360.4317664295</v>
+      </c>
+      <c r="F8">
+        <v>104098.3701427404</v>
+      </c>
+      <c r="G8">
+        <v>30642.94929025233</v>
+      </c>
+      <c r="H8">
+        <v>47242.53630801969</v>
+      </c>
+      <c r="I8">
+        <v>40973.38259634218</v>
+      </c>
+      <c r="J8">
+        <v>25022.52686608275</v>
+      </c>
+      <c r="K8">
+        <v>10477.67305055502</v>
+      </c>
+      <c r="L8">
+        <v>0</v>
+      </c>
+      <c r="M8">
+        <v>23876.44729223068</v>
+      </c>
+      <c r="N8">
+        <v>1632.724982264362</v>
+      </c>
+      <c r="O8">
+        <v>2115.615355265398</v>
+      </c>
+      <c r="P8">
+        <v>1237.406453350105</v>
+      </c>
+      <c r="Q8">
+        <v>12485.32643722762</v>
+      </c>
+      <c r="R8">
+        <v>13261.41256126442</v>
+      </c>
+      <c r="S8">
+        <v>3658.803838410196</v>
       </c>
     </row>
     <row r="9">
@@ -543,10 +907,52 @@
         <v>70504.56489624894</v>
       </c>
       <c r="D9">
-        <v>49097.30942571384</v>
+        <v>264821.0493374442</v>
       </c>
       <c r="E9">
-        <v>119590.8573778709</v>
+        <v>335289.8286197189</v>
+      </c>
+      <c r="F9">
+        <v>176295.6860130067</v>
+      </c>
+      <c r="G9">
+        <v>57323.17188569536</v>
+      </c>
+      <c r="H9">
+        <v>31202.19143874215</v>
+      </c>
+      <c r="I9">
+        <v>44555.29823806801</v>
+      </c>
+      <c r="J9">
+        <v>19564.12352579588</v>
+      </c>
+      <c r="K9">
+        <v>11143.8612438993</v>
+      </c>
+      <c r="L9">
+        <v>43908.20795814294</v>
+      </c>
+      <c r="M9">
+        <v>43293.92711892663</v>
+      </c>
+      <c r="N9">
+        <v>4622.297366525543</v>
+      </c>
+      <c r="O9">
+        <v>9207.970561648399</v>
+      </c>
+      <c r="P9">
+        <v>1603.249074683082</v>
+      </c>
+      <c r="Q9">
+        <v>17898.77467426789</v>
+      </c>
+      <c r="R9">
+        <v>30608.61711122994</v>
+      </c>
+      <c r="S9">
+        <v>7212.531025514446</v>
       </c>
     </row>
     <row r="10">
@@ -557,17 +963,59 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Ambos sexos</t>
         </is>
       </c>
       <c r="C10">
         <v>133995.4607377755</v>
       </c>
       <c r="D10">
-        <v>63386.09227244807</v>
+        <v>195826.7526571361</v>
       </c>
       <c r="E10">
-        <v>197361.1956902781</v>
+        <v>329831.4134770362</v>
+      </c>
+      <c r="F10">
+        <v>116552.9153723543</v>
+      </c>
+      <c r="G10">
+        <v>29116.58828981718</v>
+      </c>
+      <c r="H10">
+        <v>50157.24899496458</v>
+      </c>
+      <c r="I10">
+        <v>32914.33354387821</v>
+      </c>
+      <c r="J10">
+        <v>14912.24178848971</v>
+      </c>
+      <c r="K10">
+        <v>7034.411811126177</v>
+      </c>
+      <c r="L10">
+        <v>15989.78494238615</v>
+      </c>
+      <c r="M10">
+        <v>36056.51250959663</v>
+      </c>
+      <c r="N10">
+        <v>3181.058445663494</v>
+      </c>
+      <c r="O10">
+        <v>6464.572331213972</v>
+      </c>
+      <c r="P10">
+        <v>1379.972666758962</v>
+      </c>
+      <c r="Q10">
+        <v>13277.74872173246</v>
+      </c>
+      <c r="R10">
+        <v>14458.86690132577</v>
+      </c>
+      <c r="S10">
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -578,17 +1026,59 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Ambos sexos</t>
         </is>
       </c>
       <c r="C11">
         <v>119488.2122231964</v>
       </c>
       <c r="D11">
-        <v>96791.0139900051</v>
+        <v>194050.3479034956</v>
       </c>
       <c r="E11">
-        <v>216251.5274209775</v>
+        <v>313551.4133355171</v>
+      </c>
+      <c r="F11">
+        <v>81806.67082216368</v>
+      </c>
+      <c r="G11">
+        <v>41972.1828894818</v>
+      </c>
+      <c r="H11">
+        <v>70271.4941918501</v>
+      </c>
+      <c r="I11">
+        <v>38008.73813687442</v>
+      </c>
+      <c r="J11">
+        <v>5011.64978815953</v>
+      </c>
+      <c r="K11">
+        <v>5044.324364148069</v>
+      </c>
+      <c r="L11">
+        <v>11594.9609510793</v>
+      </c>
+      <c r="M11">
+        <v>17126.11661839241</v>
+      </c>
+      <c r="N11">
+        <v>1727.257427991768</v>
+      </c>
+      <c r="O11">
+        <v>3293.623535518184</v>
+      </c>
+      <c r="P11">
+        <v>1110.76604593786</v>
+      </c>
+      <c r="Q11">
+        <v>26472.19865321104</v>
+      </c>
+      <c r="R11">
+        <v>14389.2181903329</v>
+      </c>
+      <c r="S11">
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -599,17 +1089,59 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Ambos sexos</t>
         </is>
       </c>
       <c r="C12">
         <v>122507.2452801696</v>
       </c>
       <c r="D12">
-        <v>76740.94084920334</v>
+        <v>317930.7440207243</v>
       </c>
       <c r="E12">
-        <v>199255.5300144364</v>
+        <v>440477.6206734573</v>
+      </c>
+      <c r="F12">
+        <v>196662.9466162052</v>
+      </c>
+      <c r="G12">
+        <v>59525.15704836481</v>
+      </c>
+      <c r="H12">
+        <v>61742.64035615427</v>
+      </c>
+      <c r="I12">
+        <v>57604.35658292858</v>
+      </c>
+      <c r="J12">
+        <v>23810.41341521182</v>
+      </c>
+      <c r="K12">
+        <v>20360.45685048748</v>
+      </c>
+      <c r="L12">
+        <v>27250.68677264273</v>
+      </c>
+      <c r="M12">
+        <v>60737.50551927062</v>
+      </c>
+      <c r="N12">
+        <v>1260.746263852858</v>
+      </c>
+      <c r="O12">
+        <v>5638.781211811116</v>
+      </c>
+      <c r="P12">
+        <v>2072.033700758835</v>
+      </c>
+      <c r="Q12">
+        <v>14969.57753970184</v>
+      </c>
+      <c r="R12">
+        <v>33601.92292169569</v>
+      </c>
+      <c r="S12">
+        <v>8881.622886208448</v>
       </c>
     </row>
     <row r="13">
@@ -620,17 +1152,59 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Ambos sexos</t>
         </is>
       </c>
       <c r="C13">
         <v>135895.7918314252</v>
       </c>
       <c r="D13">
-        <v>108855.89043542</v>
+        <v>446804.9050784566</v>
       </c>
       <c r="E13">
-        <v>244730.6850616318</v>
+        <v>582650.2603861485</v>
+      </c>
+      <c r="F13">
+        <v>280394.0561557471</v>
+      </c>
+      <c r="G13">
+        <v>87966.1211759477</v>
+      </c>
+      <c r="H13">
+        <v>78444.72774676184</v>
+      </c>
+      <c r="I13">
+        <v>85528.68083441019</v>
+      </c>
+      <c r="J13">
+        <v>44586.65039187863</v>
+      </c>
+      <c r="K13">
+        <v>21621.53429445432</v>
+      </c>
+      <c r="L13">
+        <v>43908.20795814294</v>
+      </c>
+      <c r="M13">
+        <v>67170.37441115732</v>
+      </c>
+      <c r="N13">
+        <v>6255.022348789905</v>
+      </c>
+      <c r="O13">
+        <v>11323.5859169138</v>
+      </c>
+      <c r="P13">
+        <v>2840.655528033188</v>
+      </c>
+      <c r="Q13">
+        <v>30384.10111149551</v>
+      </c>
+      <c r="R13">
+        <v>43870.02967249435</v>
+      </c>
+      <c r="S13">
+        <v>10871.33486392464</v>
       </c>
     </row>
   </sheetData>

</xml_diff>